<commit_message>
Guard 10 · Data Integrity + Prev Close/Today Move recompute for ALL rows
Operator: '9 R2 Today Move mismatches · Current=Prev but Move≠0 · build
proper guards.'

FIX: Removed 'if status != EXIT' gate on Prev Close + Today Move recompute
in split_and_send. Now applies unconditionally to every row · derives from
row's Date + parquet · not stale carry-forward.

GUARD 10 (NEW): backend/context/data_integrity_guard.py
- Audits History row-by-row · PnL math · Today Move math · Rec date
  immutability · Entry Price immutability · Opp Age correctness
- Emits reports/context/data_integrity.json
- Hard-fails pipeline on any Today Move / PnL / immutability violation
- Wired into send flow · runs after XLSX write

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/telegram/aegis_history_india.xlsx
+++ b/reports/telegram/aegis_history_india.xlsx
@@ -6984,7 +6984,9 @@
       <c r="AK2" s="35" t="n">
         <v>24</v>
       </c>
-      <c r="AL2" s="35" t="n"/>
+      <c r="AL2" s="35" t="n">
+        <v>2398</v>
+      </c>
       <c r="AM2" s="35" t="n">
         <v>-0.59</v>
       </c>
@@ -7187,7 +7189,9 @@
       <c r="AK3" s="35" t="n">
         <v>24</v>
       </c>
-      <c r="AL3" s="35" t="n"/>
+      <c r="AL3" s="35" t="n">
+        <v>5438</v>
+      </c>
       <c r="AM3" s="35" t="n">
         <v>0.6</v>
       </c>
@@ -7390,7 +7394,9 @@
       <c r="AK4" s="36" t="n">
         <v>24</v>
       </c>
-      <c r="AL4" s="36" t="n"/>
+      <c r="AL4" s="36" t="n">
+        <v>444.8</v>
+      </c>
       <c r="AM4" s="36" t="n">
         <v>1.7</v>
       </c>
@@ -7589,7 +7595,9 @@
       <c r="AK5" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="AL5" s="37" t="n"/>
+      <c r="AL5" s="37" t="n">
+        <v>112.84</v>
+      </c>
       <c r="AM5" s="37" t="n">
         <v>0.46</v>
       </c>
@@ -7786,7 +7794,9 @@
       <c r="AK6" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="AL6" s="37" t="n"/>
+      <c r="AL6" s="37" t="n">
+        <v>414.75</v>
+      </c>
       <c r="AM6" s="37" t="n">
         <v>0.1</v>
       </c>
@@ -7983,7 +7993,9 @@
       <c r="AK7" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="AL7" s="37" t="n"/>
+      <c r="AL7" s="37" t="n">
+        <v>267.2</v>
+      </c>
       <c r="AM7" s="37" t="n">
         <v>0.49</v>
       </c>
@@ -8184,7 +8196,9 @@
       <c r="AK8" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="AL8" s="37" t="n"/>
+      <c r="AL8" s="37" t="n">
+        <v>291.9</v>
+      </c>
       <c r="AM8" s="37" t="n">
         <v>-2.42</v>
       </c>
@@ -8385,7 +8399,9 @@
       <c r="AK9" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="AL9" s="37" t="n"/>
+      <c r="AL9" s="37" t="n">
+        <v>1348.3</v>
+      </c>
       <c r="AM9" s="37" t="n">
         <v>1.13</v>
       </c>
@@ -8586,7 +8602,9 @@
       <c r="AK10" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="AL10" s="37" t="n"/>
+      <c r="AL10" s="37" t="n">
+        <v>2393.6</v>
+      </c>
       <c r="AM10" s="37" t="n">
         <v>1.91</v>
       </c>
@@ -8783,7 +8801,9 @@
       <c r="AK11" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="AL11" s="37" t="n"/>
+      <c r="AL11" s="37" t="n">
+        <v>543.2</v>
+      </c>
       <c r="AM11" s="37" t="n">
         <v>1.69</v>
       </c>
@@ -8990,7 +9010,9 @@
       <c r="AK12" s="38" t="n">
         <v>15</v>
       </c>
-      <c r="AL12" s="38" t="n"/>
+      <c r="AL12" s="38" t="n">
+        <v>425.1</v>
+      </c>
       <c r="AM12" s="38" t="n">
         <v>-0.01</v>
       </c>
@@ -9197,7 +9219,9 @@
       <c r="AK13" s="38" t="n">
         <v>15</v>
       </c>
-      <c r="AL13" s="38" t="n"/>
+      <c r="AL13" s="38" t="n">
+        <v>961.7</v>
+      </c>
       <c r="AM13" s="38" t="n">
         <v>-2.26</v>
       </c>
@@ -9404,7 +9428,9 @@
       <c r="AK14" s="38" t="n">
         <v>15</v>
       </c>
-      <c r="AL14" s="38" t="n"/>
+      <c r="AL14" s="38" t="n">
+        <v>567</v>
+      </c>
       <c r="AM14" s="38" t="n">
         <v>0.05</v>
       </c>
@@ -9595,7 +9621,9 @@
       <c r="AK15" s="39" t="n">
         <v>15</v>
       </c>
-      <c r="AL15" s="39" t="n"/>
+      <c r="AL15" s="39" t="n">
+        <v>7465</v>
+      </c>
       <c r="AM15" s="39" t="n">
         <v>-0.14</v>
       </c>
@@ -9786,7 +9814,9 @@
       <c r="AK16" s="39" t="n">
         <v>15</v>
       </c>
-      <c r="AL16" s="39" t="n"/>
+      <c r="AL16" s="39" t="n">
+        <v>699.25</v>
+      </c>
       <c r="AM16" s="39" t="n">
         <v>1.39</v>
       </c>
@@ -9973,7 +10003,9 @@
       <c r="AK17" s="35" t="n">
         <v>15</v>
       </c>
-      <c r="AL17" s="35" t="n"/>
+      <c r="AL17" s="35" t="n">
+        <v>1942.9</v>
+      </c>
       <c r="AM17" s="35" t="n">
         <v>0.64</v>
       </c>
@@ -10168,7 +10200,9 @@
       <c r="AK18" s="35" t="n">
         <v>15</v>
       </c>
-      <c r="AL18" s="35" t="n"/>
+      <c r="AL18" s="35" t="n">
+        <v>1448.3</v>
+      </c>
       <c r="AM18" s="35" t="n">
         <v>0.08</v>
       </c>
@@ -10363,7 +10397,9 @@
       <c r="AK19" s="35" t="n">
         <v>15</v>
       </c>
-      <c r="AL19" s="35" t="n"/>
+      <c r="AL19" s="35" t="n">
+        <v>1633.8</v>
+      </c>
       <c r="AM19" s="35" t="n">
         <v>0.53</v>
       </c>
@@ -10558,7 +10594,9 @@
       <c r="AK20" s="35" t="n">
         <v>15</v>
       </c>
-      <c r="AL20" s="35" t="n"/>
+      <c r="AL20" s="35" t="n">
+        <v>347.55</v>
+      </c>
       <c r="AM20" s="35" t="n">
         <v>-0.09</v>
       </c>
@@ -10749,7 +10787,9 @@
       <c r="AK21" s="36" t="n">
         <v>15</v>
       </c>
-      <c r="AL21" s="36" t="n"/>
+      <c r="AL21" s="36" t="n">
+        <v>392.7</v>
+      </c>
       <c r="AM21" s="36" t="n">
         <v>1.09</v>
       </c>
@@ -10940,7 +10980,9 @@
       <c r="AK22" s="36" t="n">
         <v>15</v>
       </c>
-      <c r="AL22" s="36" t="n"/>
+      <c r="AL22" s="36" t="n">
+        <v>382.25</v>
+      </c>
       <c r="AM22" s="36" t="n">
         <v>-0.17</v>
       </c>
@@ -11131,7 +11173,9 @@
       <c r="AK23" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="AL23" s="37" t="n"/>
+      <c r="AL23" s="37" t="n">
+        <v>501.4</v>
+      </c>
       <c r="AM23" s="37" t="n">
         <v>1.3</v>
       </c>
@@ -11326,7 +11370,9 @@
       <c r="AK24" s="36" t="n">
         <v>15</v>
       </c>
-      <c r="AL24" s="36" t="n"/>
+      <c r="AL24" s="36" t="n">
+        <v>390.3</v>
+      </c>
       <c r="AM24" s="36" t="n">
         <v>-0.12</v>
       </c>
@@ -11517,7 +11563,9 @@
       <c r="AK25" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="AL25" s="37" t="n"/>
+      <c r="AL25" s="37" t="n">
+        <v>5452</v>
+      </c>
       <c r="AM25" s="37" t="n">
         <v>0.05</v>
       </c>
@@ -11726,7 +11774,9 @@
       <c r="AK26" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="AL26" s="37" t="n"/>
+      <c r="AL26" s="37" t="n">
+        <v>2439.4</v>
+      </c>
       <c r="AM26" s="37" t="n">
         <v>0.84</v>
       </c>
@@ -11939,7 +11989,9 @@
       <c r="AK27" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="AL27" s="37" t="n"/>
+      <c r="AL27" s="37" t="n">
+        <v>1363.6</v>
+      </c>
       <c r="AM27" s="37" t="n">
         <v>0.46</v>
       </c>
@@ -12148,7 +12200,9 @@
       <c r="AK28" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="AL28" s="37" t="n"/>
+      <c r="AL28" s="37" t="n">
+        <v>11486</v>
+      </c>
       <c r="AM28" s="37" t="n">
         <v>0.99</v>
       </c>
@@ -12359,7 +12413,9 @@
       <c r="AK29" s="39" t="n">
         <v>15</v>
       </c>
-      <c r="AL29" s="39" t="n"/>
+      <c r="AL29" s="39" t="n">
+        <v>6807</v>
+      </c>
       <c r="AM29" s="39" t="n">
         <v>-0.2</v>
       </c>
@@ -12558,7 +12614,9 @@
       <c r="AK30" s="39" t="n">
         <v>15</v>
       </c>
-      <c r="AL30" s="39" t="n"/>
+      <c r="AL30" s="39" t="n">
+        <v>841.9</v>
+      </c>
       <c r="AM30" s="39" t="n">
         <v>0.37</v>
       </c>
@@ -12759,7 +12817,9 @@
       <c r="AK31" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="AL31" s="37" t="n"/>
+      <c r="AL31" s="37" t="n">
+        <v>5470.5</v>
+      </c>
       <c r="AM31" s="37" t="n">
         <v>1.42</v>
       </c>
@@ -12970,7 +13030,9 @@
       <c r="AK32" s="39" t="n">
         <v>15</v>
       </c>
-      <c r="AL32" s="39" t="n"/>
+      <c r="AL32" s="39" t="n">
+        <v>374</v>
+      </c>
       <c r="AM32" s="39" t="n">
         <v>0.8</v>
       </c>
@@ -13169,7 +13231,9 @@
       <c r="AK33" s="39" t="n">
         <v>15</v>
       </c>
-      <c r="AL33" s="39" t="n"/>
+      <c r="AL33" s="39" t="n">
+        <v>450.55</v>
+      </c>
       <c r="AM33" s="39" t="n">
         <v>-0.12</v>
       </c>
@@ -13368,12 +13432,14 @@
       <c r="AK34" s="39" t="n">
         <v>15</v>
       </c>
-      <c r="AL34" s="39" t="n"/>
+      <c r="AL34" s="39" t="n">
+        <v>397.25</v>
+      </c>
       <c r="AM34" s="39" t="n">
         <v>-1.5</v>
       </c>
       <c r="AN34" s="39" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AO34" s="39" t="n">
         <v>0</v>
@@ -13565,7 +13631,9 @@
       <c r="AK35" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="AL35" s="37" t="n"/>
+      <c r="AL35" s="37" t="n">
+        <v>11538</v>
+      </c>
       <c r="AM35" s="37" t="n">
         <v>-0.55</v>
       </c>
@@ -13776,12 +13844,14 @@
       <c r="AK36" s="39" t="n">
         <v>15</v>
       </c>
-      <c r="AL36" s="39" t="n"/>
+      <c r="AL36" s="39" t="n">
+        <v>1333</v>
+      </c>
       <c r="AM36" s="39" t="n">
         <v>-0.4</v>
       </c>
       <c r="AN36" s="39" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AO36" s="39" t="n">
         <v>0</v>
@@ -13975,7 +14045,9 @@
       <c r="AK37" s="39" t="n">
         <v>15</v>
       </c>
-      <c r="AL37" s="39" t="n"/>
+      <c r="AL37" s="39" t="n">
+        <v>2783.7</v>
+      </c>
       <c r="AM37" s="39" t="n">
         <v>-1.42</v>
       </c>
@@ -14174,7 +14246,9 @@
       <c r="AK38" s="39" t="n">
         <v>15</v>
       </c>
-      <c r="AL38" s="39" t="n"/>
+      <c r="AL38" s="39" t="n">
+        <v>1629.9</v>
+      </c>
       <c r="AM38" s="39" t="n">
         <v>-2.14</v>
       </c>
@@ -14365,7 +14439,9 @@
       <c r="AK39" s="35" t="n">
         <v>15</v>
       </c>
-      <c r="AL39" s="35" t="n"/>
+      <c r="AL39" s="35" t="n">
+        <v>1449.5</v>
+      </c>
       <c r="AM39" s="35" t="n">
         <v>0.35</v>
       </c>
@@ -14564,7 +14640,9 @@
       <c r="AK40" s="35" t="n">
         <v>15</v>
       </c>
-      <c r="AL40" s="35" t="n"/>
+      <c r="AL40" s="35" t="n">
+        <v>1955.3</v>
+      </c>
       <c r="AM40" s="35" t="n">
         <v>0.44</v>
       </c>
@@ -14763,7 +14841,9 @@
       <c r="AK41" s="35" t="n">
         <v>15</v>
       </c>
-      <c r="AL41" s="35" t="n"/>
+      <c r="AL41" s="35" t="n">
+        <v>1642.5</v>
+      </c>
       <c r="AM41" s="35" t="n">
         <v>-1.37</v>
       </c>
@@ -14962,7 +15042,9 @@
       <c r="AK42" s="35" t="n">
         <v>15</v>
       </c>
-      <c r="AL42" s="35" t="n"/>
+      <c r="AL42" s="35" t="n">
+        <v>2383.9</v>
+      </c>
       <c r="AM42" s="35" t="n">
         <v>1.09</v>
       </c>
@@ -15161,7 +15243,9 @@
       <c r="AK43" s="35" t="n">
         <v>15</v>
       </c>
-      <c r="AL43" s="35" t="n"/>
+      <c r="AL43" s="35" t="n">
+        <v>347.25</v>
+      </c>
       <c r="AM43" s="35" t="n">
         <v>-1.04</v>
       </c>
@@ -15356,7 +15440,9 @@
       <c r="AK44" s="36" t="n">
         <v>15</v>
       </c>
-      <c r="AL44" s="36" t="n"/>
+      <c r="AL44" s="36" t="n">
+        <v>397</v>
+      </c>
       <c r="AM44" s="36" t="n">
         <v>0.25</v>
       </c>
@@ -15555,7 +15641,9 @@
       <c r="AK45" s="36" t="n">
         <v>15</v>
       </c>
-      <c r="AL45" s="36" t="n"/>
+      <c r="AL45" s="36" t="n">
+        <v>285.85</v>
+      </c>
       <c r="AM45" s="36" t="n">
         <v>-0.86</v>
       </c>
@@ -15746,7 +15834,9 @@
       <c r="AK46" s="36" t="n">
         <v>15</v>
       </c>
-      <c r="AL46" s="36" t="n"/>
+      <c r="AL46" s="36" t="n">
+        <v>284.85</v>
+      </c>
       <c r="AM46" s="36" t="n">
         <v>1.46</v>
       </c>
@@ -15945,7 +16035,9 @@
       <c r="AK47" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="AL47" s="37" t="n"/>
+      <c r="AL47" s="37" t="n">
+        <v>507.9</v>
+      </c>
       <c r="AM47" s="37" t="n">
         <v>0.46</v>
       </c>
@@ -16144,7 +16236,9 @@
       <c r="AK48" s="36" t="n">
         <v>15</v>
       </c>
-      <c r="AL48" s="36" t="n"/>
+      <c r="AL48" s="36" t="n">
+        <v>389.85</v>
+      </c>
       <c r="AM48" s="36" t="n">
         <v>0.42</v>
       </c>
@@ -16339,7 +16433,9 @@
       <c r="AK49" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="AL49" s="37" t="n"/>
+      <c r="AL49" s="37" t="n">
+        <v>5454.5</v>
+      </c>
       <c r="AM49" s="37" t="n">
         <v>0.43</v>
       </c>
@@ -16538,7 +16634,9 @@
       <c r="AK50" s="36" t="n">
         <v>15</v>
       </c>
-      <c r="AL50" s="36" t="n"/>
+      <c r="AL50" s="36" t="n">
+        <v>415.15</v>
+      </c>
       <c r="AM50" s="36" t="n">
         <v>0.59</v>
       </c>
@@ -16743,7 +16841,9 @@
       <c r="AK51" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="AL51" s="37" t="n"/>
+      <c r="AL51" s="37" t="n">
+        <v>127.5</v>
+      </c>
       <c r="AM51" s="37" t="n">
         <v>1.33</v>
       </c>
@@ -16952,7 +17052,9 @@
       <c r="AK52" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="AL52" s="37" t="n"/>
+      <c r="AL52" s="37" t="n">
+        <v>5485</v>
+      </c>
       <c r="AM52" s="37" t="n">
         <v>0.26</v>
       </c>
@@ -17161,7 +17263,9 @@
       <c r="AK53" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="AL53" s="37" t="n"/>
+      <c r="AL53" s="37" t="n">
+        <v>1165.1</v>
+      </c>
       <c r="AM53" s="37" t="n">
         <v>0.21</v>
       </c>
@@ -17374,7 +17478,9 @@
       <c r="AK54" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="AL54" s="37" t="n"/>
+      <c r="AL54" s="37" t="n">
+        <v>452.35</v>
+      </c>
       <c r="AM54" s="37" t="n">
         <v>0.5</v>
       </c>
@@ -17587,7 +17693,9 @@
       <c r="AK55" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="AL55" s="37" t="n"/>
+      <c r="AL55" s="37" t="n">
+        <v>284.85</v>
+      </c>
       <c r="AM55" s="37" t="n">
         <v>1.46</v>
       </c>
@@ -17796,7 +17904,9 @@
       <c r="AK56" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="AL56" s="37" t="n"/>
+      <c r="AL56" s="37" t="n">
+        <v>2200.5</v>
+      </c>
       <c r="AM56" s="37" t="n">
         <v>-0.25</v>
       </c>
@@ -18005,7 +18115,9 @@
       <c r="AK57" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="AL57" s="37" t="n"/>
+      <c r="AL57" s="37" t="n">
+        <v>1405.3</v>
+      </c>
       <c r="AM57" s="37" t="n">
         <v>-1.52</v>
       </c>
@@ -18672,9 +18784,11 @@
       <c r="AK60" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="AL60" s="37" t="n"/>
+      <c r="AL60" s="37" t="n">
+        <v>129.2</v>
+      </c>
       <c r="AM60" s="37" t="n">
-        <v>1.33</v>
+        <v>0.32</v>
       </c>
       <c r="AN60" s="37" t="n">
         <v>-2.62</v>
@@ -18885,9 +18999,11 @@
       <c r="AK61" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="AL61" s="37" t="n"/>
+      <c r="AL61" s="37" t="n">
+        <v>5499</v>
+      </c>
       <c r="AM61" s="37" t="n">
-        <v>0.26</v>
+        <v>0.61</v>
       </c>
       <c r="AN61" s="37" t="n">
         <v>3.95</v>
@@ -19753,9 +19869,11 @@
       <c r="AK65" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="AL65" s="37" t="n"/>
+      <c r="AL65" s="37" t="n">
+        <v>454.6</v>
+      </c>
       <c r="AM65" s="37" t="n">
-        <v>0.5</v>
+        <v>1.09</v>
       </c>
       <c r="AN65" s="37" t="n">
         <v>3.65</v>
@@ -19970,9 +20088,11 @@
       <c r="AK66" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="AL66" s="37" t="n"/>
+      <c r="AL66" s="37" t="n">
+        <v>289</v>
+      </c>
       <c r="AM66" s="37" t="n">
-        <v>1.46</v>
+        <v>-1.11</v>
       </c>
       <c r="AN66" s="37" t="n">
         <v>1.03</v>
@@ -20183,9 +20303,11 @@
       <c r="AK67" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="AL67" s="37" t="n"/>
+      <c r="AL67" s="37" t="n">
+        <v>11475</v>
+      </c>
       <c r="AM67" s="37" t="n">
-        <v>-0.55</v>
+        <v>-0.17</v>
       </c>
       <c r="AN67" s="37" t="n">
         <v>2.96</v>
@@ -20609,9 +20731,11 @@
       <c r="AK69" s="37" t="n">
         <v>15</v>
       </c>
-      <c r="AL69" s="37" t="n"/>
+      <c r="AL69" s="37" t="n">
+        <v>1384</v>
+      </c>
       <c r="AM69" s="37" t="n">
-        <v>-1.52</v>
+        <v>-0.4</v>
       </c>
       <c r="AN69" s="37" t="n">
         <v>1.32</v>
@@ -21041,7 +21165,9 @@
       <c r="AK71" s="39" t="n">
         <v>15</v>
       </c>
-      <c r="AL71" s="39" t="n"/>
+      <c r="AL71" s="39" t="n">
+        <v>482</v>
+      </c>
       <c r="AM71" s="39" t="n">
         <v>-2.24</v>
       </c>
@@ -21249,7 +21375,7 @@
         <v>6.46</v>
       </c>
       <c r="AN72" s="35" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AO72" s="35" t="n">
         <v>0</v>
@@ -24685,10 +24811,10 @@
         <v>27.72</v>
       </c>
       <c r="AL90" s="35" t="n">
-        <v>2460</v>
+        <v>2421.9</v>
       </c>
       <c r="AM90" s="35" t="n">
-        <v>-1.55</v>
+        <v>1.27</v>
       </c>
       <c r="AN90" s="35" t="n">
         <v>4.31</v>
@@ -24906,10 +25032,10 @@
         <v>31.3</v>
       </c>
       <c r="AL91" s="36" t="n">
-        <v>11600</v>
+        <v>11727</v>
       </c>
       <c r="AM91" s="36" t="n">
-        <v>1.09</v>
+        <v>0.67</v>
       </c>
       <c r="AN91" s="36" t="n">
         <v>6.59</v>
@@ -25115,10 +25241,10 @@
         <v>15</v>
       </c>
       <c r="AL92" s="37" t="n">
-        <v>2410</v>
+        <v>2390.4</v>
       </c>
       <c r="AM92" s="37" t="n">
-        <v>-0.8100000000000001</v>
+        <v>-1.13</v>
       </c>
       <c r="AN92" s="37" t="n">
         <v>-2.21</v>
@@ -25318,10 +25444,10 @@
         <v>15</v>
       </c>
       <c r="AL93" s="37" t="n">
-        <v>454.6</v>
+        <v>459.55</v>
       </c>
       <c r="AM93" s="37" t="n">
-        <v>1.09</v>
+        <v>-1.93</v>
       </c>
       <c r="AN93" s="37" t="n">
         <v>1.66</v>
@@ -25521,10 +25647,10 @@
         <v>15</v>
       </c>
       <c r="AL94" s="37" t="n">
-        <v>113.99</v>
+        <v>113.54</v>
       </c>
       <c r="AM94" s="37" t="n">
-        <v>-0.39</v>
+        <v>1.12</v>
       </c>
       <c r="AN94" s="37" t="n">
         <v>1.28</v>
@@ -25724,10 +25850,10 @@
         <v>15</v>
       </c>
       <c r="AL95" s="37" t="n">
-        <v>417.6</v>
+        <v>414.05</v>
       </c>
       <c r="AM95" s="37" t="n">
-        <v>-0.85</v>
+        <v>0.29</v>
       </c>
       <c r="AN95" s="37" t="n">
         <v>0.96</v>
@@ -25927,10 +26053,10 @@
         <v>15</v>
       </c>
       <c r="AL96" s="37" t="n">
-        <v>289</v>
+        <v>285.8</v>
       </c>
       <c r="AM96" s="37" t="n">
-        <v>-1.11</v>
+        <v>0.1</v>
       </c>
       <c r="AN96" s="37" t="n">
         <v>1.13</v>
@@ -26130,10 +26256,10 @@
         <v>15</v>
       </c>
       <c r="AL97" s="37" t="n">
-        <v>562.9</v>
+        <v>597.55</v>
       </c>
       <c r="AM97" s="37" t="n">
-        <v>6.16</v>
+        <v>0.91</v>
       </c>
       <c r="AN97" s="37" t="n">
         <v>9.16</v>
@@ -26329,10 +26455,10 @@
         <v>15</v>
       </c>
       <c r="AL98" s="37" t="n">
-        <v>129.2</v>
+        <v>129.61</v>
       </c>
       <c r="AM98" s="37" t="n">
-        <v>0.32</v>
+        <v>-1.94</v>
       </c>
       <c r="AN98" s="37" t="n">
         <v>-4.51</v>
@@ -26528,10 +26654,10 @@
         <v>15</v>
       </c>
       <c r="AL99" s="37" t="n">
-        <v>5499</v>
+        <v>5532.5</v>
       </c>
       <c r="AM99" s="37" t="n">
-        <v>0.61</v>
+        <v>-1.04</v>
       </c>
       <c r="AN99" s="37" t="n">
         <v>2.87</v>
@@ -26727,10 +26853,10 @@
         <v>15</v>
       </c>
       <c r="AL100" s="37" t="n">
-        <v>11475</v>
+        <v>11456</v>
       </c>
       <c r="AM100" s="37" t="n">
-        <v>-0.17</v>
+        <v>-1.68</v>
       </c>
       <c r="AN100" s="37" t="n">
         <v>1.22</v>
@@ -26926,10 +27052,10 @@
         <v>15</v>
       </c>
       <c r="AL101" s="37" t="n">
-        <v>1384</v>
+        <v>1378.5</v>
       </c>
       <c r="AM101" s="37" t="n">
-        <v>-0.4</v>
+        <v>-0.44</v>
       </c>
       <c r="AN101" s="37" t="n">
         <v>0.87</v>
@@ -27129,10 +27255,10 @@
         <v>15</v>
       </c>
       <c r="AL102" s="37" t="n">
-        <v>1454.6</v>
+        <v>1449.6</v>
       </c>
       <c r="AM102" s="37" t="n">
-        <v>-0.34</v>
+        <v>-1.97</v>
       </c>
       <c r="AN102" s="37" t="n">
         <v>-1.22</v>
@@ -27332,10 +27458,10 @@
         <v>15</v>
       </c>
       <c r="AL103" s="37" t="n">
-        <v>1964</v>
+        <v>1949</v>
       </c>
       <c r="AM103" s="37" t="n">
-        <v>-0.76</v>
+        <v>-0.21</v>
       </c>
       <c r="AN103" s="37" t="n">
         <v>-3.46</v>
@@ -27535,10 +27661,10 @@
         <v>15</v>
       </c>
       <c r="AL104" s="37" t="n">
-        <v>2410</v>
+        <v>2390.4</v>
       </c>
       <c r="AM104" s="37" t="n">
-        <v>-0.8100000000000001</v>
+        <v>-1.13</v>
       </c>
       <c r="AN104" s="37" t="n">
         <v>-2.21</v>
@@ -27738,10 +27864,10 @@
         <v>15</v>
       </c>
       <c r="AL105" s="37" t="n">
-        <v>1620</v>
+        <v>1657</v>
       </c>
       <c r="AM105" s="37" t="n">
-        <v>2.28</v>
+        <v>0.18</v>
       </c>
       <c r="AN105" s="37" t="n">
         <v>2.12</v>
@@ -27941,10 +28067,10 @@
         <v>15</v>
       </c>
       <c r="AL106" s="37" t="n">
-        <v>343.65</v>
+        <v>346.9</v>
       </c>
       <c r="AM106" s="37" t="n">
-        <v>0.95</v>
+        <v>-1.27</v>
       </c>
       <c r="AN106" s="37" t="n">
         <v>-0.9399999999999999</v>
@@ -28140,10 +28266,10 @@
         <v>15</v>
       </c>
       <c r="AL107" s="37" t="n">
-        <v>398</v>
+        <v>397.2</v>
       </c>
       <c r="AM107" s="37" t="n">
-        <v>-0.2</v>
+        <v>-1.62</v>
       </c>
       <c r="AN107" s="37" t="n">
         <v>0.37</v>
@@ -28343,10 +28469,10 @@
         <v>15</v>
       </c>
       <c r="AL108" s="37" t="n">
-        <v>283.4</v>
+        <v>276.8</v>
       </c>
       <c r="AM108" s="37" t="n">
-        <v>-2.33</v>
+        <v>-1.88</v>
       </c>
       <c r="AN108" s="37" t="n">
         <v>-5</v>
@@ -28542,10 +28668,10 @@
         <v>15</v>
       </c>
       <c r="AL109" s="37" t="n">
-        <v>510.25</v>
+        <v>510.85</v>
       </c>
       <c r="AM109" s="37" t="n">
-        <v>0.12</v>
+        <v>1.78</v>
       </c>
       <c r="AN109" s="37" t="n">
         <v>5.18</v>
@@ -28745,10 +28871,10 @@
         <v>15</v>
       </c>
       <c r="AL110" s="37" t="n">
-        <v>391.5</v>
+        <v>390.05</v>
       </c>
       <c r="AM110" s="37" t="n">
-        <v>-0.37</v>
+        <v>2.81</v>
       </c>
       <c r="AN110" s="37" t="n">
         <v>3.16</v>
@@ -28948,10 +29074,10 @@
         <v>15</v>
       </c>
       <c r="AL111" s="37" t="n">
-        <v>417.6</v>
+        <v>414.05</v>
       </c>
       <c r="AM111" s="37" t="n">
-        <v>-0.85</v>
+        <v>0.29</v>
       </c>
       <c r="AN111" s="37" t="n">
         <v>0.96</v>
@@ -29147,10 +29273,10 @@
         <v>15</v>
       </c>
       <c r="AL112" s="37" t="n">
-        <v>5478</v>
+        <v>5429</v>
       </c>
       <c r="AM112" s="37" t="n">
-        <v>-0.89</v>
+        <v>1.49</v>
       </c>
       <c r="AN112" s="37" t="n">
         <v>1.92</v>
@@ -29350,10 +29476,10 @@
         <v>15</v>
       </c>
       <c r="AL113" s="37" t="n">
-        <v>380</v>
+        <v>378.9</v>
       </c>
       <c r="AM113" s="37" t="n">
-        <v>-0.29</v>
+        <v>0.44</v>
       </c>
       <c r="AN113" s="37" t="n">
         <v>-0.28</v>
@@ -29557,10 +29683,10 @@
         <v>24</v>
       </c>
       <c r="AL114" s="35" t="n">
-        <v>519.75</v>
+        <v>553.3</v>
       </c>
       <c r="AM114" s="35" t="n">
-        <v>6.46</v>
+        <v>-3.22</v>
       </c>
       <c r="AN114" s="35" t="n">
         <v>-3.22</v>
@@ -29762,10 +29888,10 @@
         <v>8.550000000000001</v>
       </c>
       <c r="AL115" s="36" t="n">
-        <v>289</v>
+        <v>285.8</v>
       </c>
       <c r="AM115" s="36" t="n">
-        <v>-1.11</v>
+        <v>0.1</v>
       </c>
       <c r="AN115" s="36" t="n">
         <v>1.13</v>
@@ -29951,7 +30077,7 @@
         </is>
       </c>
       <c r="AB116" s="38" t="n">
-        <v>853.4</v>
+        <v>889.5</v>
       </c>
       <c r="AC116" s="38" t="n">
         <v>845</v>
@@ -29981,13 +30107,13 @@
         <v>15</v>
       </c>
       <c r="AL116" s="38" t="n">
-        <v>845</v>
+        <v>853.4</v>
       </c>
       <c r="AM116" s="38" t="n">
-        <v>0.99</v>
+        <v>4.23</v>
       </c>
       <c r="AN116" s="38" t="n">
-        <v>0.99</v>
+        <v>5.27</v>
       </c>
       <c r="AO116" s="38" t="n">
         <v>0</v>
@@ -30172,7 +30298,7 @@
         </is>
       </c>
       <c r="AB117" s="38" t="n">
-        <v>6834</v>
+        <v>6774</v>
       </c>
       <c r="AC117" s="38" t="n">
         <v>6793.5</v>
@@ -30202,13 +30328,13 @@
         <v>15</v>
       </c>
       <c r="AL117" s="38" t="n">
-        <v>6793.5</v>
+        <v>6834</v>
       </c>
       <c r="AM117" s="38" t="n">
-        <v>0.6</v>
+        <v>-0.88</v>
       </c>
       <c r="AN117" s="38" t="n">
-        <v>0.6</v>
+        <v>-0.29</v>
       </c>
       <c r="AO117" s="38" t="n">
         <v>0</v>
@@ -30393,7 +30519,7 @@
         </is>
       </c>
       <c r="AB118" s="38" t="n">
-        <v>443.9</v>
+        <v>442.8</v>
       </c>
       <c r="AC118" s="38" t="n">
         <v>450</v>
@@ -30423,13 +30549,13 @@
         <v>15</v>
       </c>
       <c r="AL118" s="38" t="n">
-        <v>450</v>
+        <v>443.9</v>
       </c>
       <c r="AM118" s="38" t="n">
-        <v>-1.36</v>
+        <v>-0.25</v>
       </c>
       <c r="AN118" s="38" t="n">
-        <v>-1.36</v>
+        <v>-1.6</v>
       </c>
       <c r="AO118" s="38" t="n">
         <v>0</v>
@@ -30602,7 +30728,7 @@
         </is>
       </c>
       <c r="AB119" s="38" t="n">
-        <v>471.2</v>
+        <v>473.3</v>
       </c>
       <c r="AC119" s="38" t="n">
         <v>471.2</v>
@@ -30632,13 +30758,13 @@
         <v>15</v>
       </c>
       <c r="AL119" s="38" t="n">
-        <v>482</v>
+        <v>471.2</v>
       </c>
       <c r="AM119" s="38" t="n">
-        <v>-2.24</v>
+        <v>0.45</v>
       </c>
       <c r="AN119" s="38" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="AO119" s="38" t="n">
         <v>0</v>
@@ -30811,7 +30937,7 @@
         </is>
       </c>
       <c r="AB120" s="38" t="n">
-        <v>1594.5</v>
+        <v>1584.8</v>
       </c>
       <c r="AC120" s="38" t="n">
         <v>1595</v>
@@ -30841,13 +30967,13 @@
         <v>15</v>
       </c>
       <c r="AL120" s="38" t="n">
-        <v>1595</v>
+        <v>1594.5</v>
       </c>
       <c r="AM120" s="38" t="n">
-        <v>-0.03</v>
+        <v>-0.61</v>
       </c>
       <c r="AN120" s="38" t="n">
-        <v>-0.03</v>
+        <v>-0.64</v>
       </c>
       <c r="AO120" s="38" t="n">
         <v>0</v>
@@ -31020,7 +31146,7 @@
         </is>
       </c>
       <c r="AB121" s="38" t="n">
-        <v>1296.8</v>
+        <v>1285</v>
       </c>
       <c r="AC121" s="38" t="n">
         <v>1327.7</v>
@@ -31050,13 +31176,13 @@
         <v>15</v>
       </c>
       <c r="AL121" s="38" t="n">
-        <v>1327.7</v>
+        <v>1296.8</v>
       </c>
       <c r="AM121" s="38" t="n">
-        <v>-2.33</v>
+        <v>-0.91</v>
       </c>
       <c r="AN121" s="38" t="n">
-        <v>-2.33</v>
+        <v>-3.22</v>
       </c>
       <c r="AO121" s="38" t="n">
         <v>0</v>
@@ -31245,10 +31371,10 @@
         <v>15</v>
       </c>
       <c r="AL122" s="37" t="n">
-        <v>7395</v>
+        <v>7531.5</v>
       </c>
       <c r="AM122" s="37" t="n">
-        <v>1.85</v>
+        <v>-1.28</v>
       </c>
       <c r="AN122" s="37" t="n">
         <v>-0.26</v>
@@ -31448,10 +31574,10 @@
         <v>15</v>
       </c>
       <c r="AL123" s="37" t="n">
-        <v>709.55</v>
+        <v>731</v>
       </c>
       <c r="AM123" s="37" t="n">
-        <v>3.02</v>
+        <v>-1.44</v>
       </c>
       <c r="AN123" s="37" t="n">
         <v>1.62</v>
@@ -31639,10 +31765,10 @@
         <v>15</v>
       </c>
       <c r="AL124" s="37" t="n">
-        <v>377</v>
+        <v>380.35</v>
       </c>
       <c r="AM124" s="37" t="n">
-        <v>0.89</v>
+        <v>0.17</v>
       </c>
       <c r="AN124" s="37" t="n">
         <v>1.06</v>
@@ -31834,10 +31960,10 @@
         <v>15</v>
       </c>
       <c r="AL125" s="37" t="n">
-        <v>391.3</v>
+        <v>387.9</v>
       </c>
       <c r="AM125" s="37" t="n">
-        <v>-0.87</v>
+        <v>1.57</v>
       </c>
       <c r="AN125" s="37" t="n">
         <v>0.6899999999999999</v>
@@ -32025,10 +32151,10 @@
         <v>15</v>
       </c>
       <c r="AL126" s="37" t="n">
-        <v>2744.3</v>
+        <v>2764.2</v>
       </c>
       <c r="AM126" s="37" t="n">
-        <v>0.73</v>
+        <v>0.28</v>
       </c>
       <c r="AN126" s="37" t="n">
         <v>1.01</v>
@@ -32244,10 +32370,10 @@
         <v>29.35</v>
       </c>
       <c r="AL127" s="35" t="n">
-        <v>2421.9</v>
+        <v>2452.7</v>
       </c>
       <c r="AM127" s="35" t="n">
-        <v>1.27</v>
+        <v>0</v>
       </c>
       <c r="AN127" s="35" t="n">
         <v>4.31</v>
@@ -32276,7 +32402,7 @@
       </c>
       <c r="AU127" s="35" t="inlineStr">
         <is>
-          <t>2026-08-10 05:40</t>
+          <t>2026-08-10 05:58</t>
         </is>
       </c>
       <c r="AV127" s="35" t="inlineStr">
@@ -32461,10 +32587,10 @@
         <v>20.01</v>
       </c>
       <c r="AL128" s="35" t="n">
-        <v>553.3</v>
+        <v>535.5</v>
       </c>
       <c r="AM128" s="35" t="n">
-        <v>-3.22</v>
+        <v>0</v>
       </c>
       <c r="AN128" s="35" t="n">
         <v>-3.22</v>
@@ -32493,7 +32619,7 @@
       </c>
       <c r="AU128" s="35" t="inlineStr">
         <is>
-          <t>2026-08-10 05:40</t>
+          <t>2026-08-10 05:58</t>
         </is>
       </c>
       <c r="AV128" s="35" t="inlineStr">
@@ -32682,10 +32808,10 @@
         <v>32.17</v>
       </c>
       <c r="AL129" s="36" t="n">
-        <v>11727</v>
+        <v>11805</v>
       </c>
       <c r="AM129" s="36" t="n">
-        <v>0.67</v>
+        <v>0</v>
       </c>
       <c r="AN129" s="36" t="n">
         <v>6.59</v>
@@ -32714,7 +32840,7 @@
       </c>
       <c r="AU129" s="36" t="inlineStr">
         <is>
-          <t>2026-08-10 05:40</t>
+          <t>2026-08-10 05:58</t>
         </is>
       </c>
       <c r="AV129" s="36" t="inlineStr">
@@ -32905,10 +33031,10 @@
         <v>15</v>
       </c>
       <c r="AL130" s="38" t="n">
-        <v>128.5</v>
+        <v>131.95</v>
       </c>
       <c r="AM130" s="38" t="n">
-        <v>2.68</v>
+        <v>0</v>
       </c>
       <c r="AN130" s="38" t="n">
         <v>0</v>
@@ -33108,10 +33234,10 @@
         <v>15</v>
       </c>
       <c r="AL131" s="38" t="n">
-        <v>176.1</v>
+        <v>183.6</v>
       </c>
       <c r="AM131" s="38" t="n">
-        <v>4.26</v>
+        <v>0</v>
       </c>
       <c r="AN131" s="38" t="n">
         <v>0</v>
@@ -33311,10 +33437,10 @@
         <v>15</v>
       </c>
       <c r="AL132" s="38" t="n">
-        <v>5020.5</v>
+        <v>4924</v>
       </c>
       <c r="AM132" s="38" t="n">
-        <v>-1.92</v>
+        <v>0</v>
       </c>
       <c r="AN132" s="38" t="n">
         <v>0</v>
@@ -33522,10 +33648,10 @@
         <v>15</v>
       </c>
       <c r="AL133" s="38" t="n">
-        <v>7531.5</v>
+        <v>7435</v>
       </c>
       <c r="AM133" s="38" t="n">
-        <v>-1.28</v>
+        <v>0</v>
       </c>
       <c r="AN133" s="38" t="n">
         <v>-0.26</v>
@@ -33717,10 +33843,10 @@
         <v>11.35</v>
       </c>
       <c r="AL134" s="35" t="n">
-        <v>1449.6</v>
+        <v>1421</v>
       </c>
       <c r="AM134" s="35" t="n">
-        <v>-1.97</v>
+        <v>0</v>
       </c>
       <c r="AN134" s="35" t="n">
         <v>-1.22</v>
@@ -33922,10 +34048,10 @@
         <v>8.02</v>
       </c>
       <c r="AL135" s="35" t="n">
-        <v>1949</v>
+        <v>1945</v>
       </c>
       <c r="AM135" s="35" t="n">
-        <v>-0.21</v>
+        <v>0</v>
       </c>
       <c r="AN135" s="35" t="n">
         <v>-3.46</v>
@@ -34127,10 +34253,10 @@
         <v>10.78</v>
       </c>
       <c r="AL136" s="35" t="n">
-        <v>1657</v>
+        <v>1660</v>
       </c>
       <c r="AM136" s="35" t="n">
-        <v>0.18</v>
+        <v>0</v>
       </c>
       <c r="AN136" s="35" t="n">
         <v>2.12</v>
@@ -34332,10 +34458,10 @@
         <v>13</v>
       </c>
       <c r="AL137" s="35" t="n">
-        <v>2390.4</v>
+        <v>2363.5</v>
       </c>
       <c r="AM137" s="35" t="n">
-        <v>-1.13</v>
+        <v>0</v>
       </c>
       <c r="AN137" s="35" t="n">
         <v>-2.21</v>
@@ -34537,10 +34663,10 @@
         <v>16.01</v>
       </c>
       <c r="AL138" s="35" t="n">
-        <v>397.2</v>
+        <v>390.75</v>
       </c>
       <c r="AM138" s="35" t="n">
-        <v>-1.62</v>
+        <v>0</v>
       </c>
       <c r="AN138" s="35" t="n">
         <v>0.37</v>
@@ -34742,10 +34868,10 @@
         <v>14.47</v>
       </c>
       <c r="AL139" s="36" t="n">
-        <v>346.9</v>
+        <v>342.5</v>
       </c>
       <c r="AM139" s="36" t="n">
-        <v>-1.27</v>
+        <v>0</v>
       </c>
       <c r="AN139" s="36" t="n">
         <v>-0.9399999999999999</v>
@@ -34943,10 +35069,10 @@
         <v>19.22</v>
       </c>
       <c r="AL140" s="36" t="n">
-        <v>390.05</v>
+        <v>401</v>
       </c>
       <c r="AM140" s="36" t="n">
-        <v>2.81</v>
+        <v>0</v>
       </c>
       <c r="AN140" s="36" t="n">
         <v>3.16</v>
@@ -35152,10 +35278,10 @@
         <v>9.779999999999999</v>
       </c>
       <c r="AL141" s="36" t="n">
-        <v>276.8</v>
+        <v>271.6</v>
       </c>
       <c r="AM141" s="36" t="n">
-        <v>-1.88</v>
+        <v>0</v>
       </c>
       <c r="AN141" s="36" t="n">
         <v>-5</v>
@@ -35353,10 +35479,10 @@
         <v>21.56</v>
       </c>
       <c r="AL142" s="37" t="n">
-        <v>510.85</v>
+        <v>519.95</v>
       </c>
       <c r="AM142" s="37" t="n">
-        <v>1.78</v>
+        <v>0</v>
       </c>
       <c r="AN142" s="37" t="n">
         <v>5.18</v>
@@ -35554,10 +35680,10 @@
         <v>8.550000000000001</v>
       </c>
       <c r="AL143" s="36" t="n">
-        <v>285.8</v>
+        <v>286.1</v>
       </c>
       <c r="AM143" s="36" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="AN143" s="36" t="n">
         <v>1.13</v>
@@ -35582,7 +35708,7 @@
       </c>
       <c r="AU143" s="36" t="inlineStr">
         <is>
-          <t>2026-08-10 05:40</t>
+          <t>2026-08-10 05:58</t>
         </is>
       </c>
       <c r="AV143" s="36" t="inlineStr">
@@ -35759,10 +35885,10 @@
         <v>16.66</v>
       </c>
       <c r="AL144" s="36" t="n">
-        <v>414.05</v>
+        <v>415.25</v>
       </c>
       <c r="AM144" s="36" t="n">
-        <v>0.29</v>
+        <v>0</v>
       </c>
       <c r="AN144" s="36" t="n">
         <v>0.96</v>
@@ -35960,10 +36086,10 @@
         <v>17.78</v>
       </c>
       <c r="AL145" s="37" t="n">
-        <v>5429</v>
+        <v>5510</v>
       </c>
       <c r="AM145" s="37" t="n">
-        <v>1.49</v>
+        <v>0</v>
       </c>
       <c r="AN145" s="37" t="n">
         <v>1.92</v>
@@ -36165,10 +36291,10 @@
         <v>15</v>
       </c>
       <c r="AL146" s="37" t="n">
-        <v>2390.4</v>
+        <v>2363.5</v>
       </c>
       <c r="AM146" s="37" t="n">
-        <v>-1.13</v>
+        <v>0</v>
       </c>
       <c r="AN146" s="37" t="n">
         <v>-2.21</v>
@@ -36191,7 +36317,7 @@
       </c>
       <c r="AU146" s="37" t="inlineStr">
         <is>
-          <t>2026-08-10 05:40</t>
+          <t>2026-08-10 05:58</t>
         </is>
       </c>
       <c r="AV146" s="37" t="inlineStr">
@@ -36368,10 +36494,10 @@
         <v>15</v>
       </c>
       <c r="AL147" s="37" t="n">
-        <v>459.55</v>
+        <v>450.7</v>
       </c>
       <c r="AM147" s="37" t="n">
-        <v>-1.93</v>
+        <v>0</v>
       </c>
       <c r="AN147" s="37" t="n">
         <v>1.66</v>
@@ -36394,7 +36520,7 @@
       </c>
       <c r="AU147" s="37" t="inlineStr">
         <is>
-          <t>2026-08-10 05:40</t>
+          <t>2026-08-10 05:58</t>
         </is>
       </c>
       <c r="AV147" s="37" t="inlineStr">
@@ -36571,10 +36697,10 @@
         <v>15</v>
       </c>
       <c r="AL148" s="37" t="n">
-        <v>113.54</v>
+        <v>114.81</v>
       </c>
       <c r="AM148" s="37" t="n">
-        <v>1.12</v>
+        <v>0</v>
       </c>
       <c r="AN148" s="37" t="n">
         <v>1.28</v>
@@ -36597,7 +36723,7 @@
       </c>
       <c r="AU148" s="37" t="inlineStr">
         <is>
-          <t>2026-08-10 05:40</t>
+          <t>2026-08-10 05:58</t>
         </is>
       </c>
       <c r="AV148" s="37" t="inlineStr">
@@ -36774,10 +36900,10 @@
         <v>15</v>
       </c>
       <c r="AL149" s="37" t="n">
-        <v>414.05</v>
+        <v>415.25</v>
       </c>
       <c r="AM149" s="37" t="n">
-        <v>0.29</v>
+        <v>0</v>
       </c>
       <c r="AN149" s="37" t="n">
         <v>0.96</v>
@@ -36800,7 +36926,7 @@
       </c>
       <c r="AU149" s="37" t="inlineStr">
         <is>
-          <t>2026-08-10 05:40</t>
+          <t>2026-08-10 05:58</t>
         </is>
       </c>
       <c r="AV149" s="37" t="inlineStr">
@@ -36977,10 +37103,10 @@
         <v>15</v>
       </c>
       <c r="AL150" s="37" t="n">
-        <v>285.8</v>
+        <v>286.1</v>
       </c>
       <c r="AM150" s="37" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="AN150" s="37" t="n">
         <v>1.13</v>
@@ -37003,7 +37129,7 @@
       </c>
       <c r="AU150" s="37" t="inlineStr">
         <is>
-          <t>2026-08-10 05:40</t>
+          <t>2026-08-10 05:58</t>
         </is>
       </c>
       <c r="AV150" s="37" t="inlineStr">
@@ -37180,10 +37306,10 @@
         <v>15</v>
       </c>
       <c r="AL151" s="37" t="n">
-        <v>597.55</v>
+        <v>603</v>
       </c>
       <c r="AM151" s="37" t="n">
-        <v>0.91</v>
+        <v>0</v>
       </c>
       <c r="AN151" s="37" t="n">
         <v>9.16</v>
@@ -37206,7 +37332,7 @@
       </c>
       <c r="AU151" s="37" t="inlineStr">
         <is>
-          <t>2026-08-10 05:40</t>
+          <t>2026-08-10 05:58</t>
         </is>
       </c>
       <c r="AV151" s="37" t="inlineStr">
@@ -37383,10 +37509,10 @@
         <v>15</v>
       </c>
       <c r="AL152" s="37" t="n">
-        <v>731</v>
+        <v>720.5</v>
       </c>
       <c r="AM152" s="37" t="n">
-        <v>-1.44</v>
+        <v>0</v>
       </c>
       <c r="AN152" s="37" t="n">
         <v>1.62</v>
@@ -37409,7 +37535,7 @@
       </c>
       <c r="AU152" s="37" t="inlineStr">
         <is>
-          <t>2026-08-10 05:40</t>
+          <t>2026-08-10 05:58</t>
         </is>
       </c>
       <c r="AV152" s="37" t="inlineStr">
@@ -37578,10 +37704,10 @@
         <v>15</v>
       </c>
       <c r="AL153" s="37" t="n">
-        <v>129.61</v>
+        <v>127.1</v>
       </c>
       <c r="AM153" s="37" t="n">
-        <v>-1.94</v>
+        <v>0</v>
       </c>
       <c r="AN153" s="37" t="n">
         <v>-4.51</v>
@@ -37604,7 +37730,7 @@
       </c>
       <c r="AU153" s="37" t="inlineStr">
         <is>
-          <t>2026-08-10 05:40</t>
+          <t>2026-08-10 05:58</t>
         </is>
       </c>
       <c r="AV153" s="37" t="inlineStr">
@@ -37777,10 +37903,10 @@
         <v>15</v>
       </c>
       <c r="AL154" s="37" t="n">
-        <v>5532.5</v>
+        <v>5475</v>
       </c>
       <c r="AM154" s="37" t="n">
-        <v>-1.04</v>
+        <v>0</v>
       </c>
       <c r="AN154" s="37" t="n">
         <v>2.87</v>
@@ -37803,7 +37929,7 @@
       </c>
       <c r="AU154" s="37" t="inlineStr">
         <is>
-          <t>2026-08-10 05:40</t>
+          <t>2026-08-10 05:58</t>
         </is>
       </c>
       <c r="AV154" s="37" t="inlineStr">
@@ -37976,10 +38102,10 @@
         <v>15</v>
       </c>
       <c r="AL155" s="37" t="n">
-        <v>11456</v>
+        <v>11263</v>
       </c>
       <c r="AM155" s="37" t="n">
-        <v>-1.68</v>
+        <v>0</v>
       </c>
       <c r="AN155" s="37" t="n">
         <v>1.22</v>
@@ -38002,7 +38128,7 @@
       </c>
       <c r="AU155" s="37" t="inlineStr">
         <is>
-          <t>2026-08-10 05:40</t>
+          <t>2026-08-10 05:58</t>
         </is>
       </c>
       <c r="AV155" s="37" t="inlineStr">
@@ -38175,10 +38301,10 @@
         <v>15</v>
       </c>
       <c r="AL156" s="37" t="n">
-        <v>1378.5</v>
+        <v>1372.4</v>
       </c>
       <c r="AM156" s="37" t="n">
-        <v>-0.44</v>
+        <v>0</v>
       </c>
       <c r="AN156" s="37" t="n">
         <v>0.87</v>
@@ -38201,7 +38327,7 @@
       </c>
       <c r="AU156" s="37" t="inlineStr">
         <is>
-          <t>2026-08-10 05:40</t>
+          <t>2026-08-10 05:58</t>
         </is>
       </c>
       <c r="AV156" s="37" t="inlineStr">
@@ -38370,10 +38496,10 @@
         <v>15</v>
       </c>
       <c r="AL157" s="37" t="n">
-        <v>380.35</v>
+        <v>381</v>
       </c>
       <c r="AM157" s="37" t="n">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="AN157" s="37" t="n">
         <v>1.06</v>
@@ -38396,7 +38522,7 @@
       </c>
       <c r="AU157" s="37" t="inlineStr">
         <is>
-          <t>2026-08-10 05:40</t>
+          <t>2026-08-10 05:58</t>
         </is>
       </c>
       <c r="AV157" s="37" t="inlineStr">
@@ -38565,10 +38691,10 @@
         <v>15</v>
       </c>
       <c r="AL158" s="37" t="n">
-        <v>387.9</v>
+        <v>394</v>
       </c>
       <c r="AM158" s="37" t="n">
-        <v>1.57</v>
+        <v>0</v>
       </c>
       <c r="AN158" s="37" t="n">
         <v>0.6899999999999999</v>
@@ -38591,7 +38717,7 @@
       </c>
       <c r="AU158" s="37" t="inlineStr">
         <is>
-          <t>2026-08-10 05:40</t>
+          <t>2026-08-10 05:58</t>
         </is>
       </c>
       <c r="AV158" s="37" t="inlineStr">
@@ -38756,10 +38882,10 @@
         <v>15</v>
       </c>
       <c r="AL159" s="37" t="n">
-        <v>2764.2</v>
+        <v>2772</v>
       </c>
       <c r="AM159" s="37" t="n">
-        <v>0.28</v>
+        <v>0</v>
       </c>
       <c r="AN159" s="37" t="n">
         <v>1.01</v>
@@ -38782,7 +38908,7 @@
       </c>
       <c r="AU159" s="37" t="inlineStr">
         <is>
-          <t>2026-08-10 05:40</t>
+          <t>2026-08-10 05:58</t>
         </is>
       </c>
       <c r="AV159" s="37" t="inlineStr">
@@ -38959,10 +39085,10 @@
         <v>15</v>
       </c>
       <c r="AL160" s="37" t="n">
-        <v>1449.6</v>
+        <v>1421</v>
       </c>
       <c r="AM160" s="37" t="n">
-        <v>-1.97</v>
+        <v>0</v>
       </c>
       <c r="AN160" s="37" t="n">
         <v>-1.22</v>
@@ -38985,7 +39111,7 @@
       </c>
       <c r="AU160" s="37" t="inlineStr">
         <is>
-          <t>2026-08-10 05:40</t>
+          <t>2026-08-10 05:58</t>
         </is>
       </c>
       <c r="AV160" s="37" t="inlineStr">
@@ -39162,10 +39288,10 @@
         <v>15</v>
       </c>
       <c r="AL161" s="37" t="n">
-        <v>1949</v>
+        <v>1945</v>
       </c>
       <c r="AM161" s="37" t="n">
-        <v>-0.21</v>
+        <v>0</v>
       </c>
       <c r="AN161" s="37" t="n">
         <v>-3.46</v>
@@ -39188,7 +39314,7 @@
       </c>
       <c r="AU161" s="37" t="inlineStr">
         <is>
-          <t>2026-08-10 05:40</t>
+          <t>2026-08-10 05:58</t>
         </is>
       </c>
       <c r="AV161" s="37" t="inlineStr">
@@ -39365,10 +39491,10 @@
         <v>15</v>
       </c>
       <c r="AL162" s="37" t="n">
-        <v>2390.4</v>
+        <v>2363.5</v>
       </c>
       <c r="AM162" s="37" t="n">
-        <v>-1.13</v>
+        <v>0</v>
       </c>
       <c r="AN162" s="37" t="n">
         <v>-2.21</v>
@@ -39391,7 +39517,7 @@
       </c>
       <c r="AU162" s="37" t="inlineStr">
         <is>
-          <t>2026-08-10 05:40</t>
+          <t>2026-08-10 05:58</t>
         </is>
       </c>
       <c r="AV162" s="37" t="inlineStr">
@@ -39568,10 +39694,10 @@
         <v>15</v>
       </c>
       <c r="AL163" s="37" t="n">
-        <v>1657</v>
+        <v>1660</v>
       </c>
       <c r="AM163" s="37" t="n">
-        <v>0.18</v>
+        <v>0</v>
       </c>
       <c r="AN163" s="37" t="n">
         <v>2.12</v>
@@ -39594,7 +39720,7 @@
       </c>
       <c r="AU163" s="37" t="inlineStr">
         <is>
-          <t>2026-08-10 05:40</t>
+          <t>2026-08-10 05:58</t>
         </is>
       </c>
       <c r="AV163" s="37" t="inlineStr">
@@ -39771,10 +39897,10 @@
         <v>15</v>
       </c>
       <c r="AL164" s="37" t="n">
-        <v>346.9</v>
+        <v>342.5</v>
       </c>
       <c r="AM164" s="37" t="n">
-        <v>-1.27</v>
+        <v>0</v>
       </c>
       <c r="AN164" s="37" t="n">
         <v>-0.9399999999999999</v>
@@ -39797,7 +39923,7 @@
       </c>
       <c r="AU164" s="37" t="inlineStr">
         <is>
-          <t>2026-08-10 05:40</t>
+          <t>2026-08-10 05:58</t>
         </is>
       </c>
       <c r="AV164" s="37" t="inlineStr">
@@ -39970,10 +40096,10 @@
         <v>15</v>
       </c>
       <c r="AL165" s="37" t="n">
-        <v>397.2</v>
+        <v>390.75</v>
       </c>
       <c r="AM165" s="37" t="n">
-        <v>-1.62</v>
+        <v>0</v>
       </c>
       <c r="AN165" s="37" t="n">
         <v>0.37</v>
@@ -39996,7 +40122,7 @@
       </c>
       <c r="AU165" s="37" t="inlineStr">
         <is>
-          <t>2026-08-10 05:40</t>
+          <t>2026-08-10 05:58</t>
         </is>
       </c>
       <c r="AV165" s="37" t="inlineStr">
@@ -40173,10 +40299,10 @@
         <v>15</v>
       </c>
       <c r="AL166" s="37" t="n">
-        <v>276.8</v>
+        <v>271.6</v>
       </c>
       <c r="AM166" s="37" t="n">
-        <v>-1.88</v>
+        <v>0</v>
       </c>
       <c r="AN166" s="37" t="n">
         <v>-5</v>
@@ -40199,7 +40325,7 @@
       </c>
       <c r="AU166" s="37" t="inlineStr">
         <is>
-          <t>2026-08-10 05:40</t>
+          <t>2026-08-10 05:58</t>
         </is>
       </c>
       <c r="AV166" s="37" t="inlineStr">
@@ -40372,10 +40498,10 @@
         <v>15</v>
       </c>
       <c r="AL167" s="37" t="n">
-        <v>510.85</v>
+        <v>519.95</v>
       </c>
       <c r="AM167" s="37" t="n">
-        <v>1.78</v>
+        <v>0</v>
       </c>
       <c r="AN167" s="37" t="n">
         <v>5.18</v>
@@ -40398,7 +40524,7 @@
       </c>
       <c r="AU167" s="37" t="inlineStr">
         <is>
-          <t>2026-08-10 05:40</t>
+          <t>2026-08-10 05:58</t>
         </is>
       </c>
       <c r="AV167" s="37" t="inlineStr">
@@ -40575,10 +40701,10 @@
         <v>15</v>
       </c>
       <c r="AL168" s="37" t="n">
-        <v>390.05</v>
+        <v>401</v>
       </c>
       <c r="AM168" s="37" t="n">
-        <v>2.81</v>
+        <v>0</v>
       </c>
       <c r="AN168" s="37" t="n">
         <v>3.16</v>
@@ -40601,7 +40727,7 @@
       </c>
       <c r="AU168" s="37" t="inlineStr">
         <is>
-          <t>2026-08-10 05:40</t>
+          <t>2026-08-10 05:58</t>
         </is>
       </c>
       <c r="AV168" s="37" t="inlineStr">
@@ -40778,10 +40904,10 @@
         <v>15</v>
       </c>
       <c r="AL169" s="37" t="n">
-        <v>414.05</v>
+        <v>415.25</v>
       </c>
       <c r="AM169" s="37" t="n">
-        <v>0.29</v>
+        <v>0</v>
       </c>
       <c r="AN169" s="37" t="n">
         <v>0.96</v>
@@ -40804,7 +40930,7 @@
       </c>
       <c r="AU169" s="37" t="inlineStr">
         <is>
-          <t>2026-08-10 05:40</t>
+          <t>2026-08-10 05:58</t>
         </is>
       </c>
       <c r="AV169" s="37" t="inlineStr">
@@ -40977,10 +41103,10 @@
         <v>15</v>
       </c>
       <c r="AL170" s="37" t="n">
-        <v>5429</v>
+        <v>5510</v>
       </c>
       <c r="AM170" s="37" t="n">
-        <v>1.49</v>
+        <v>0</v>
       </c>
       <c r="AN170" s="37" t="n">
         <v>1.92</v>
@@ -41003,7 +41129,7 @@
       </c>
       <c r="AU170" s="37" t="inlineStr">
         <is>
-          <t>2026-08-10 05:40</t>
+          <t>2026-08-10 05:58</t>
         </is>
       </c>
       <c r="AV170" s="37" t="inlineStr">
@@ -41180,10 +41306,10 @@
         <v>15</v>
       </c>
       <c r="AL171" s="37" t="n">
-        <v>378.9</v>
+        <v>380.55</v>
       </c>
       <c r="AM171" s="37" t="n">
-        <v>0.44</v>
+        <v>0</v>
       </c>
       <c r="AN171" s="37" t="n">
         <v>-0.28</v>
@@ -41206,7 +41332,7 @@
       </c>
       <c r="AU171" s="37" t="inlineStr">
         <is>
-          <t>2026-08-10 05:40</t>
+          <t>2026-08-10 05:58</t>
         </is>
       </c>
       <c r="AV171" s="37" t="inlineStr">

</xml_diff>